<commit_message>
feat: catalogo APERTURA (BO-A/CL-C3/BR-F/FD-S/FD-T) 17 items + 6 procedimientos + motivos actualizados desde manuales Trutzschler
</commit_message>
<xml_diff>
--- a/public/Catalogo.xlsx
+++ b/public/Catalogo.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9398" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9602" uniqueCount="632">
   <si>
     <t>Marca</t>
   </si>
@@ -1730,6 +1730,189 @@
   </si>
   <si>
     <t>Para transporte</t>
+  </si>
+  <si>
+    <t>BO-A</t>
+  </si>
+  <si>
+    <t>019</t>
+  </si>
+  <si>
+    <t>CORREA TRAPEZOIDAL DIN7753-XPA 1000</t>
+  </si>
+  <si>
+    <t>037181753740</t>
+  </si>
+  <si>
+    <t>1 año</t>
+  </si>
+  <si>
+    <t>Sustitucion anual</t>
+  </si>
+  <si>
+    <t>CORREA TRAPEZOIDAL DIN7753-XPA 910</t>
+  </si>
+  <si>
+    <t>037181753719</t>
+  </si>
+  <si>
+    <t>ELEVACION</t>
+  </si>
+  <si>
+    <t>ELEVAC</t>
+  </si>
+  <si>
+    <t>CABLES METALICOS</t>
+  </si>
+  <si>
+    <t>2 años</t>
+  </si>
+  <si>
+    <t>Sustituir ambos cables</t>
+  </si>
+  <si>
+    <t>ELECTRONICA</t>
+  </si>
+  <si>
+    <t>ELECTRON</t>
+  </si>
+  <si>
+    <t>PILA ZPB4 / KSZ5</t>
+  </si>
+  <si>
+    <t>Sustitucion segun aviso</t>
+  </si>
+  <si>
+    <t>DEPOSITO DE GRASA</t>
+  </si>
+  <si>
+    <t>Desmontar para mantenimiento</t>
+  </si>
+  <si>
+    <t>CL-C3</t>
+  </si>
+  <si>
+    <t>ALIMENTACION</t>
+  </si>
+  <si>
+    <t>097</t>
+  </si>
+  <si>
+    <t>CORREA DE TRANSMISION</t>
+  </si>
+  <si>
+    <t>Comprobar tension y desgaste</t>
+  </si>
+  <si>
+    <t>SISTEMA ELECTRICO</t>
+  </si>
+  <si>
+    <t>ELECTRICO</t>
+  </si>
+  <si>
+    <t>FUSIBLES ARMARIO DE MANDO</t>
+  </si>
+  <si>
+    <t>Sustituir en caso de fallo</t>
+  </si>
+  <si>
+    <t>MODULO EEPROM</t>
+  </si>
+  <si>
+    <t>Sustitucion por reparacion</t>
+  </si>
+  <si>
+    <t>ESTANQUIDAD</t>
+  </si>
+  <si>
+    <t>ESTANQ</t>
+  </si>
+  <si>
+    <t>TIRA DE ESTANQUIDAD</t>
+  </si>
+  <si>
+    <t>Desmontar/Montar segun desgaste</t>
+  </si>
+  <si>
+    <t>BR-F/FD</t>
+  </si>
+  <si>
+    <t>ACCIONAMIENTO</t>
+  </si>
+  <si>
+    <t>ACCIONAM</t>
+  </si>
+  <si>
+    <t>109</t>
+  </si>
+  <si>
+    <t>COJINETE DEL VENTILADOR</t>
+  </si>
+  <si>
+    <t>Sustituir por desgaste</t>
+  </si>
+  <si>
+    <t>COJINETE DEL MOTOR</t>
+  </si>
+  <si>
+    <t>SISTEMA NEUMATICO</t>
+  </si>
+  <si>
+    <t>PALETA DEL VENTILADOR</t>
+  </si>
+  <si>
+    <t>Comprobar estado/limpieza</t>
+  </si>
+  <si>
+    <t>FD-S</t>
+  </si>
+  <si>
+    <t>250</t>
+  </si>
+  <si>
+    <t>CORREA TRAPEZOIDAL</t>
+  </si>
+  <si>
+    <t>Ajustar tension</t>
+  </si>
+  <si>
+    <t>CADENA DE RODILLOS</t>
+  </si>
+  <si>
+    <t>Comprobar tension</t>
+  </si>
+  <si>
+    <t>MODULO DE MEMORIA</t>
+  </si>
+  <si>
+    <t>Sustituir en reparacion</t>
+  </si>
+  <si>
+    <t>FD-T</t>
+  </si>
+  <si>
+    <t>SENSORES</t>
+  </si>
+  <si>
+    <t>988</t>
+  </si>
+  <si>
+    <t>BARRERA DE LUZ</t>
+  </si>
+  <si>
+    <t>Control de llenado</t>
+  </si>
+  <si>
+    <t>ESTRUCTURA</t>
+  </si>
+  <si>
+    <t>ESTRUCT</t>
+  </si>
+  <si>
+    <t>TOLVA DE LLENADO</t>
+  </si>
+  <si>
+    <t>Limpieza periodica</t>
   </si>
 </sst>
 </file>
@@ -2156,7 +2339,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L824"/>
+  <dimension ref="A1:L841"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="9.140625"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -32032,6 +32215,652 @@
         <v>570</v>
       </c>
     </row>
+    <row r="825" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A825" t="s">
+        <v>492</v>
+      </c>
+      <c r="B825" t="s">
+        <v>571</v>
+      </c>
+      <c r="C825" t="s">
+        <v>19</v>
+      </c>
+      <c r="D825" t="s">
+        <v>527</v>
+      </c>
+      <c r="E825" t="s">
+        <v>528</v>
+      </c>
+      <c r="F825" t="s">
+        <v>572</v>
+      </c>
+      <c r="G825" t="s">
+        <v>18</v>
+      </c>
+      <c r="H825" t="s">
+        <v>573</v>
+      </c>
+      <c r="I825" t="s">
+        <v>18</v>
+      </c>
+      <c r="J825" t="s">
+        <v>574</v>
+      </c>
+      <c r="K825" t="s">
+        <v>575</v>
+      </c>
+      <c r="L825" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="826" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A826" t="s">
+        <v>492</v>
+      </c>
+      <c r="B826" t="s">
+        <v>571</v>
+      </c>
+      <c r="C826" t="s">
+        <v>19</v>
+      </c>
+      <c r="D826" t="s">
+        <v>527</v>
+      </c>
+      <c r="E826" t="s">
+        <v>528</v>
+      </c>
+      <c r="F826" t="s">
+        <v>572</v>
+      </c>
+      <c r="G826" t="s">
+        <v>18</v>
+      </c>
+      <c r="H826" t="s">
+        <v>577</v>
+      </c>
+      <c r="I826" t="s">
+        <v>18</v>
+      </c>
+      <c r="J826" t="s">
+        <v>578</v>
+      </c>
+      <c r="K826" t="s">
+        <v>575</v>
+      </c>
+      <c r="L826" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="827" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A827" t="s">
+        <v>492</v>
+      </c>
+      <c r="B827" t="s">
+        <v>571</v>
+      </c>
+      <c r="C827" t="s">
+        <v>19</v>
+      </c>
+      <c r="D827" t="s">
+        <v>579</v>
+      </c>
+      <c r="E827" t="s">
+        <v>580</v>
+      </c>
+      <c r="F827" t="s">
+        <v>572</v>
+      </c>
+      <c r="G827" t="s">
+        <v>18</v>
+      </c>
+      <c r="H827" t="s">
+        <v>581</v>
+      </c>
+      <c r="I827" t="s">
+        <v>18</v>
+      </c>
+      <c r="J827" t="s">
+        <v>18</v>
+      </c>
+      <c r="K827" t="s">
+        <v>582</v>
+      </c>
+      <c r="L827" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="828" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A828" t="s">
+        <v>492</v>
+      </c>
+      <c r="B828" t="s">
+        <v>571</v>
+      </c>
+      <c r="C828" t="s">
+        <v>19</v>
+      </c>
+      <c r="D828" t="s">
+        <v>584</v>
+      </c>
+      <c r="E828" t="s">
+        <v>585</v>
+      </c>
+      <c r="F828" t="s">
+        <v>572</v>
+      </c>
+      <c r="G828" t="s">
+        <v>18</v>
+      </c>
+      <c r="H828" t="s">
+        <v>586</v>
+      </c>
+      <c r="I828" t="s">
+        <v>18</v>
+      </c>
+      <c r="J828" t="s">
+        <v>18</v>
+      </c>
+      <c r="K828" t="s">
+        <v>19</v>
+      </c>
+      <c r="L828" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="829" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A829" t="s">
+        <v>492</v>
+      </c>
+      <c r="B829" t="s">
+        <v>571</v>
+      </c>
+      <c r="C829" t="s">
+        <v>19</v>
+      </c>
+      <c r="D829" t="s">
+        <v>539</v>
+      </c>
+      <c r="E829" t="s">
+        <v>540</v>
+      </c>
+      <c r="F829" t="s">
+        <v>572</v>
+      </c>
+      <c r="G829" t="s">
+        <v>18</v>
+      </c>
+      <c r="H829" t="s">
+        <v>588</v>
+      </c>
+      <c r="I829" t="s">
+        <v>18</v>
+      </c>
+      <c r="J829" t="s">
+        <v>18</v>
+      </c>
+      <c r="K829" t="s">
+        <v>19</v>
+      </c>
+      <c r="L829" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="830" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A830" t="s">
+        <v>492</v>
+      </c>
+      <c r="B830" t="s">
+        <v>590</v>
+      </c>
+      <c r="C830" t="s">
+        <v>19</v>
+      </c>
+      <c r="D830" t="s">
+        <v>591</v>
+      </c>
+      <c r="E830" t="s">
+        <v>496</v>
+      </c>
+      <c r="F830" t="s">
+        <v>592</v>
+      </c>
+      <c r="G830" t="s">
+        <v>18</v>
+      </c>
+      <c r="H830" t="s">
+        <v>593</v>
+      </c>
+      <c r="I830" t="s">
+        <v>18</v>
+      </c>
+      <c r="J830" t="s">
+        <v>18</v>
+      </c>
+      <c r="K830" t="s">
+        <v>19</v>
+      </c>
+      <c r="L830" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="831" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A831" t="s">
+        <v>492</v>
+      </c>
+      <c r="B831" t="s">
+        <v>590</v>
+      </c>
+      <c r="C831" t="s">
+        <v>19</v>
+      </c>
+      <c r="D831" t="s">
+        <v>595</v>
+      </c>
+      <c r="E831" t="s">
+        <v>596</v>
+      </c>
+      <c r="F831" t="s">
+        <v>592</v>
+      </c>
+      <c r="G831" t="s">
+        <v>18</v>
+      </c>
+      <c r="H831" t="s">
+        <v>597</v>
+      </c>
+      <c r="I831" t="s">
+        <v>18</v>
+      </c>
+      <c r="J831" t="s">
+        <v>18</v>
+      </c>
+      <c r="K831" t="s">
+        <v>19</v>
+      </c>
+      <c r="L831" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="832" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A832" t="s">
+        <v>492</v>
+      </c>
+      <c r="B832" t="s">
+        <v>590</v>
+      </c>
+      <c r="C832" t="s">
+        <v>19</v>
+      </c>
+      <c r="D832" t="s">
+        <v>584</v>
+      </c>
+      <c r="E832" t="s">
+        <v>585</v>
+      </c>
+      <c r="F832" t="s">
+        <v>592</v>
+      </c>
+      <c r="G832" t="s">
+        <v>18</v>
+      </c>
+      <c r="H832" t="s">
+        <v>599</v>
+      </c>
+      <c r="I832" t="s">
+        <v>18</v>
+      </c>
+      <c r="J832" t="s">
+        <v>18</v>
+      </c>
+      <c r="K832" t="s">
+        <v>19</v>
+      </c>
+      <c r="L832" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="833" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A833" t="s">
+        <v>492</v>
+      </c>
+      <c r="B833" t="s">
+        <v>590</v>
+      </c>
+      <c r="C833" t="s">
+        <v>19</v>
+      </c>
+      <c r="D833" t="s">
+        <v>601</v>
+      </c>
+      <c r="E833" t="s">
+        <v>602</v>
+      </c>
+      <c r="F833" t="s">
+        <v>592</v>
+      </c>
+      <c r="G833" t="s">
+        <v>18</v>
+      </c>
+      <c r="H833" t="s">
+        <v>603</v>
+      </c>
+      <c r="I833" t="s">
+        <v>18</v>
+      </c>
+      <c r="J833" t="s">
+        <v>18</v>
+      </c>
+      <c r="K833" t="s">
+        <v>19</v>
+      </c>
+      <c r="L833" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="834" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A834" t="s">
+        <v>492</v>
+      </c>
+      <c r="B834" t="s">
+        <v>605</v>
+      </c>
+      <c r="C834" t="s">
+        <v>19</v>
+      </c>
+      <c r="D834" t="s">
+        <v>606</v>
+      </c>
+      <c r="E834" t="s">
+        <v>607</v>
+      </c>
+      <c r="F834" t="s">
+        <v>608</v>
+      </c>
+      <c r="G834" t="s">
+        <v>18</v>
+      </c>
+      <c r="H834" t="s">
+        <v>609</v>
+      </c>
+      <c r="I834" t="s">
+        <v>18</v>
+      </c>
+      <c r="J834" t="s">
+        <v>18</v>
+      </c>
+      <c r="K834" t="s">
+        <v>19</v>
+      </c>
+      <c r="L834" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="835" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A835" t="s">
+        <v>492</v>
+      </c>
+      <c r="B835" t="s">
+        <v>605</v>
+      </c>
+      <c r="C835" t="s">
+        <v>19</v>
+      </c>
+      <c r="D835" t="s">
+        <v>606</v>
+      </c>
+      <c r="E835" t="s">
+        <v>607</v>
+      </c>
+      <c r="F835" t="s">
+        <v>608</v>
+      </c>
+      <c r="G835" t="s">
+        <v>18</v>
+      </c>
+      <c r="H835" t="s">
+        <v>611</v>
+      </c>
+      <c r="I835" t="s">
+        <v>18</v>
+      </c>
+      <c r="J835" t="s">
+        <v>18</v>
+      </c>
+      <c r="K835" t="s">
+        <v>19</v>
+      </c>
+      <c r="L835" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="836" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A836" t="s">
+        <v>492</v>
+      </c>
+      <c r="B836" t="s">
+        <v>605</v>
+      </c>
+      <c r="C836" t="s">
+        <v>19</v>
+      </c>
+      <c r="D836" t="s">
+        <v>612</v>
+      </c>
+      <c r="E836" t="s">
+        <v>534</v>
+      </c>
+      <c r="F836" t="s">
+        <v>608</v>
+      </c>
+      <c r="G836" t="s">
+        <v>18</v>
+      </c>
+      <c r="H836" t="s">
+        <v>613</v>
+      </c>
+      <c r="I836" t="s">
+        <v>18</v>
+      </c>
+      <c r="J836" t="s">
+        <v>18</v>
+      </c>
+      <c r="K836" t="s">
+        <v>19</v>
+      </c>
+      <c r="L836" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="837" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A837" t="s">
+        <v>492</v>
+      </c>
+      <c r="B837" t="s">
+        <v>615</v>
+      </c>
+      <c r="C837" t="s">
+        <v>19</v>
+      </c>
+      <c r="D837" t="s">
+        <v>527</v>
+      </c>
+      <c r="E837" t="s">
+        <v>528</v>
+      </c>
+      <c r="F837" t="s">
+        <v>616</v>
+      </c>
+      <c r="G837" t="s">
+        <v>18</v>
+      </c>
+      <c r="H837" t="s">
+        <v>617</v>
+      </c>
+      <c r="I837" t="s">
+        <v>18</v>
+      </c>
+      <c r="J837" t="s">
+        <v>18</v>
+      </c>
+      <c r="K837" t="s">
+        <v>19</v>
+      </c>
+      <c r="L837" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="838" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A838" t="s">
+        <v>492</v>
+      </c>
+      <c r="B838" t="s">
+        <v>615</v>
+      </c>
+      <c r="C838" t="s">
+        <v>19</v>
+      </c>
+      <c r="D838" t="s">
+        <v>527</v>
+      </c>
+      <c r="E838" t="s">
+        <v>528</v>
+      </c>
+      <c r="F838" t="s">
+        <v>616</v>
+      </c>
+      <c r="G838" t="s">
+        <v>18</v>
+      </c>
+      <c r="H838" t="s">
+        <v>619</v>
+      </c>
+      <c r="I838" t="s">
+        <v>18</v>
+      </c>
+      <c r="J838" t="s">
+        <v>18</v>
+      </c>
+      <c r="K838" t="s">
+        <v>19</v>
+      </c>
+      <c r="L838" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="839" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A839" t="s">
+        <v>492</v>
+      </c>
+      <c r="B839" t="s">
+        <v>615</v>
+      </c>
+      <c r="C839" t="s">
+        <v>19</v>
+      </c>
+      <c r="D839" t="s">
+        <v>584</v>
+      </c>
+      <c r="E839" t="s">
+        <v>585</v>
+      </c>
+      <c r="F839" t="s">
+        <v>616</v>
+      </c>
+      <c r="G839" t="s">
+        <v>18</v>
+      </c>
+      <c r="H839" t="s">
+        <v>621</v>
+      </c>
+      <c r="I839" t="s">
+        <v>18</v>
+      </c>
+      <c r="J839" t="s">
+        <v>18</v>
+      </c>
+      <c r="K839" t="s">
+        <v>19</v>
+      </c>
+      <c r="L839" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="840" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A840" t="s">
+        <v>492</v>
+      </c>
+      <c r="B840" t="s">
+        <v>623</v>
+      </c>
+      <c r="C840" t="s">
+        <v>19</v>
+      </c>
+      <c r="D840" t="s">
+        <v>624</v>
+      </c>
+      <c r="E840" t="s">
+        <v>624</v>
+      </c>
+      <c r="F840" t="s">
+        <v>625</v>
+      </c>
+      <c r="G840" t="s">
+        <v>18</v>
+      </c>
+      <c r="H840" t="s">
+        <v>626</v>
+      </c>
+      <c r="I840" t="s">
+        <v>18</v>
+      </c>
+      <c r="J840" t="s">
+        <v>18</v>
+      </c>
+      <c r="K840" t="s">
+        <v>19</v>
+      </c>
+      <c r="L840" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="841" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A841" t="s">
+        <v>492</v>
+      </c>
+      <c r="B841" t="s">
+        <v>623</v>
+      </c>
+      <c r="C841" t="s">
+        <v>19</v>
+      </c>
+      <c r="D841" t="s">
+        <v>628</v>
+      </c>
+      <c r="E841" t="s">
+        <v>629</v>
+      </c>
+      <c r="F841" t="s">
+        <v>625</v>
+      </c>
+      <c r="G841" t="s">
+        <v>18</v>
+      </c>
+      <c r="H841" t="s">
+        <v>630</v>
+      </c>
+      <c r="I841" t="s">
+        <v>18</v>
+      </c>
+      <c r="J841" t="s">
+        <v>18</v>
+      </c>
+      <c r="K841" t="s">
+        <v>19</v>
+      </c>
+      <c r="L841" t="s">
+        <v>631</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L806"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>